<commit_message>
Update Excel file with new content
</commit_message>
<xml_diff>
--- a/SKU.xlsx
+++ b/SKU.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ข้อมูลในเครื่อง\D - ดาวน์โหลด\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A74488E-F3F4-4E19-9ECC-CF0A2B17C8E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7057512A-D7F6-4D1F-AA74-C0E91297248E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Sheet 1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet 1'!$A$1:$L$325</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet 1'!$A$1:$L$328</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2002" uniqueCount="741">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2004" uniqueCount="743">
   <si>
     <t>No.</t>
   </si>
@@ -2261,6 +2261,12 @@
   </si>
   <si>
     <t xml:space="preserve">	สกรูล้อ toyota/isuzu</t>
+  </si>
+  <si>
+    <t>น๊อตล้อ เบอร์19x1.25</t>
+  </si>
+  <si>
+    <t>หัวแปลงเติมลมรถเกรดเอดอร์</t>
   </si>
 </sst>
 </file>
@@ -2657,10 +2663,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L328"/>
+  <dimension ref="A1:L329"/>
   <sheetFormatPr defaultColWidth="15" defaultRowHeight="19.95" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="4" width="20" customWidth="1"/>
+    <col min="3" max="3" width="20" customWidth="1"/>
+    <col min="4" max="4" width="28.8984375" bestFit="1" customWidth="1"/>
     <col min="5" max="6" width="35" customWidth="1"/>
   </cols>
   <sheetData>
@@ -5527,7 +5534,9 @@
       <c r="C79" s="2" t="s">
         <v>539</v>
       </c>
-      <c r="D79" s="2"/>
+      <c r="D79" s="2" t="s">
+        <v>742</v>
+      </c>
       <c r="E79" s="2" t="s">
         <v>540</v>
       </c>
@@ -6909,7 +6918,9 @@
       <c r="C117" s="2" t="s">
         <v>232</v>
       </c>
-      <c r="D117" s="2"/>
+      <c r="D117" s="2" t="s">
+        <v>741</v>
+      </c>
       <c r="E117" s="2" t="s">
         <v>233</v>
       </c>
@@ -14376,8 +14387,11 @@
         <v>500</v>
       </c>
     </row>
+    <row r="329" spans="1:12" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E329" s="2"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L325" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <autoFilter ref="A1:L328" xr:uid="{00000000-0001-0000-0000-000000000000}">
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:L325">
       <sortCondition ref="B1:B325"/>
     </sortState>

</xml_diff>